<commit_message>
Added new class DataAttr to keep track of output data units and other metadata and implemented across all modules
</commit_message>
<xml_diff>
--- a/data/default/MachineryAndEnergyMgmt.xlsx
+++ b/data/default/MachineryAndEnergyMgmt.xlsx
@@ -477,7 +477,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="946" uniqueCount="335">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="949" uniqueCount="336">
   <si>
     <t>f_crop</t>
   </si>
@@ -979,9 +979,6 @@
     <t>Transport kärna</t>
   </si>
   <si>
-    <t>Transport halm</t>
-  </si>
-  <si>
     <t>Transport vagn allmän</t>
   </si>
   <si>
@@ -1660,6 +1657,12 @@
   </si>
   <si>
     <t>Natural gas</t>
+  </si>
+  <si>
+    <t>kWh/ton DM</t>
+  </si>
+  <si>
+    <t>Adjusted to dry matter. Transport halm</t>
   </si>
 </sst>
 </file>
@@ -2461,25 +2464,25 @@
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B1" s="14" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="14" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D1" s="14" t="s">
+        <v>202</v>
+      </c>
+      <c r="E1" s="14" t="s">
         <v>203</v>
       </c>
-      <c r="E1" s="14" t="s">
-        <v>204</v>
-      </c>
       <c r="F1" s="14" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="G1" s="14" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="H1" s="14" t="s">
         <v>52</v>
@@ -2491,7 +2494,7 @@
         <v>129</v>
       </c>
       <c r="K1" s="14" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="L1" s="14" t="s">
         <v>1</v>
@@ -2511,7 +2514,7 @@
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="L2" s="20" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="M2" s="9">
         <v>0</v>
@@ -2525,13 +2528,13 @@
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="L4" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="M4" s="18">
         <f>(241822577+237201100)/(241822577+237201100+5856000+8368914)*100</f>
@@ -2541,18 +2544,18 @@
         <v>128</v>
       </c>
       <c r="P4" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="L5" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="M5" s="18">
         <f>100-M4</f>
@@ -2562,18 +2565,18 @@
         <v>128</v>
       </c>
       <c r="P5" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="L6" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="M6" s="10">
         <v>0</v>
@@ -2584,13 +2587,13 @@
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="L7" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="M7" s="10">
         <v>0</v>
@@ -2606,16 +2609,16 @@
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C9" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="L9" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="M9" s="10">
         <v>100</v>
@@ -2626,10 +2629,10 @@
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C10" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G10" s="4"/>
       <c r="L10" s="6"/>
@@ -2637,16 +2640,16 @@
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C11" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="L11" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="M11" s="10">
         <v>100</v>
@@ -2657,16 +2660,16 @@
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C12" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="L12" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="M12" s="10">
         <v>100</v>
@@ -2682,19 +2685,19 @@
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C14" t="s">
+        <v>235</v>
+      </c>
+      <c r="D14" t="s">
         <v>236</v>
       </c>
-      <c r="D14" t="s">
-        <v>237</v>
-      </c>
       <c r="G14" s="4" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="L14" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="M14" s="10">
         <v>100</v>
@@ -2705,19 +2708,19 @@
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C15" t="s">
+        <v>235</v>
+      </c>
+      <c r="D15" t="s">
         <v>236</v>
       </c>
-      <c r="D15" t="s">
-        <v>237</v>
-      </c>
       <c r="G15" s="6" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="L15" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="M15" s="10">
         <v>100</v>
@@ -2728,19 +2731,19 @@
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C16" t="s">
+        <v>235</v>
+      </c>
+      <c r="D16" t="s">
         <v>236</v>
       </c>
-      <c r="D16" t="s">
-        <v>237</v>
-      </c>
       <c r="G16" s="6" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="L16" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="M16" s="10">
         <v>100</v>
@@ -2756,19 +2759,19 @@
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C18" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E18" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="L18" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="M18" s="10">
         <v>100</v>
@@ -2777,24 +2780,24 @@
         <v>128</v>
       </c>
       <c r="P18" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C19" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E19" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="L19" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="M19">
         <v>4</v>
@@ -2803,24 +2806,24 @@
         <v>128</v>
       </c>
       <c r="P19" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C20" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E20" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="L20" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="M20">
         <v>76</v>
@@ -2829,24 +2832,24 @@
         <v>128</v>
       </c>
       <c r="P20" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C21" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E21" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="L21" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="M21">
         <v>20</v>
@@ -2855,24 +2858,24 @@
         <v>128</v>
       </c>
       <c r="P21" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C22" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E22" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="L22" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="M22" s="10">
         <v>100</v>
@@ -2881,24 +2884,24 @@
         <v>128</v>
       </c>
       <c r="P22" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C23" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E23" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="L23" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="M23" s="10">
         <v>100</v>
@@ -2907,24 +2910,24 @@
         <v>128</v>
       </c>
       <c r="P23" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C24" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E24" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="L24" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="M24">
         <v>20</v>
@@ -2933,24 +2936,24 @@
         <v>128</v>
       </c>
       <c r="P24" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C25" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E25" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="G25" s="6" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="L25" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="M25">
         <v>60</v>
@@ -2959,24 +2962,24 @@
         <v>128</v>
       </c>
       <c r="P25" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C26" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E26" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="L26" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="M26">
         <v>20.000000000000018</v>
@@ -2985,24 +2988,24 @@
         <v>128</v>
       </c>
       <c r="P26" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C27" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E27" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="G27" s="6" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="L27" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="M27" s="10">
         <v>100</v>
@@ -3011,7 +3014,7 @@
         <v>128</v>
       </c>
       <c r="P27" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="28" spans="1:16" x14ac:dyDescent="0.25">
@@ -3021,13 +3024,13 @@
     </row>
     <row r="29" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>153</v>
+      </c>
+      <c r="G29" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="L29" s="6" t="s">
         <v>154</v>
-      </c>
-      <c r="G29" s="6" t="s">
-        <v>330</v>
-      </c>
-      <c r="L29" s="6" t="s">
-        <v>155</v>
       </c>
       <c r="M29" s="11">
         <v>6.4777062142923141</v>
@@ -3036,18 +3039,18 @@
         <v>128</v>
       </c>
       <c r="P29" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>153</v>
+      </c>
+      <c r="G30" s="6" t="s">
+        <v>333</v>
+      </c>
+      <c r="L30" s="6" t="s">
         <v>154</v>
-      </c>
-      <c r="G30" s="6" t="s">
-        <v>334</v>
-      </c>
-      <c r="L30" s="6" t="s">
-        <v>155</v>
       </c>
       <c r="M30" s="11">
         <v>8.7567853491111922</v>
@@ -3056,21 +3059,21 @@
         <v>128</v>
       </c>
       <c r="O30" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="P30" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
+        <v>153</v>
+      </c>
+      <c r="G31" s="6" t="s">
+        <v>330</v>
+      </c>
+      <c r="L31" s="6" t="s">
         <v>154</v>
-      </c>
-      <c r="G31" s="6" t="s">
-        <v>331</v>
-      </c>
-      <c r="L31" s="6" t="s">
-        <v>155</v>
       </c>
       <c r="M31" s="18">
         <v>59.671114354829328</v>
@@ -3079,21 +3082,21 @@
         <v>128</v>
       </c>
       <c r="O31" s="19" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="P31" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
+        <v>153</v>
+      </c>
+      <c r="G32" s="6" t="s">
+        <v>328</v>
+      </c>
+      <c r="L32" s="6" t="s">
         <v>154</v>
-      </c>
-      <c r="G32" s="6" t="s">
-        <v>329</v>
-      </c>
-      <c r="L32" s="6" t="s">
-        <v>155</v>
       </c>
       <c r="M32" s="18">
         <v>16.802918820320372</v>
@@ -3104,13 +3107,13 @@
     </row>
     <row r="33" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
+        <v>153</v>
+      </c>
+      <c r="G33" s="6" t="s">
+        <v>332</v>
+      </c>
+      <c r="L33" s="6" t="s">
         <v>154</v>
-      </c>
-      <c r="G33" s="6" t="s">
-        <v>333</v>
-      </c>
-      <c r="L33" s="6" t="s">
-        <v>155</v>
       </c>
       <c r="M33" s="11">
         <v>7.4851294970113242</v>
@@ -3121,13 +3124,13 @@
     </row>
     <row r="34" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
+        <v>153</v>
+      </c>
+      <c r="G34" s="6" t="s">
+        <v>331</v>
+      </c>
+      <c r="L34" s="6" t="s">
         <v>154</v>
-      </c>
-      <c r="G34" s="6" t="s">
-        <v>332</v>
-      </c>
-      <c r="L34" s="6" t="s">
-        <v>155</v>
       </c>
       <c r="M34" s="11">
         <v>0.80634576443547301</v>
@@ -3180,7 +3183,7 @@
     </row>
     <row r="39" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B39" s="1"/>
       <c r="C39" s="1"/>
@@ -3201,14 +3204,14 @@
     <row r="40" spans="1:16" x14ac:dyDescent="0.25">
       <c r="G40" s="4"/>
       <c r="L40" s="9" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="M40" s="23">
         <v>0</v>
       </c>
       <c r="N40" s="9"/>
       <c r="O40" s="9" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="41" spans="1:16" x14ac:dyDescent="0.25">
@@ -3217,377 +3220,377 @@
     </row>
     <row r="42" spans="1:16" x14ac:dyDescent="0.25">
       <c r="G42" s="4" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="K42" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="L42" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="M42" s="18">
         <f>74100</f>
         <v>74100</v>
       </c>
       <c r="N42" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="O42" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="P42" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="43" spans="1:16" x14ac:dyDescent="0.25">
       <c r="G43" s="4" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="K43" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="L43" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="M43" s="11">
         <f>3.9</f>
         <v>3.9</v>
       </c>
       <c r="N43" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="P43" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="44" spans="1:16" x14ac:dyDescent="0.25">
       <c r="G44" s="4" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="K44" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="L44" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="M44" s="11">
         <f>3.9</f>
         <v>3.9</v>
       </c>
       <c r="N44" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="P44" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="45" spans="1:16" x14ac:dyDescent="0.25">
       <c r="G45" s="4" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="K45" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="L45" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="M45" s="18">
         <v>0</v>
       </c>
       <c r="N45" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="46" spans="1:16" x14ac:dyDescent="0.25">
       <c r="G46" s="4" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="K46" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="L46" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="M46" s="22">
         <f t="shared" ref="M46:M47" si="0">M43</f>
         <v>3.9</v>
       </c>
       <c r="N46" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="O46" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="47" spans="1:16" x14ac:dyDescent="0.25">
       <c r="G47" s="4" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="K47" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="L47" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="M47" s="22">
         <f t="shared" si="0"/>
         <v>3.9</v>
       </c>
       <c r="N47" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="O47" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="48" spans="1:16" x14ac:dyDescent="0.25">
       <c r="G48" s="6" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="K48" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="L48" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="M48" s="18">
         <v>73300</v>
       </c>
       <c r="N48" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="O48" t="s">
+        <v>189</v>
+      </c>
+      <c r="P48" t="s">
         <v>190</v>
-      </c>
-      <c r="P48" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="49" spans="1:16" x14ac:dyDescent="0.25">
       <c r="G49" s="6" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="K49" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="L49" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="M49">
         <v>10</v>
       </c>
       <c r="N49" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="P49" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="50" spans="1:16" x14ac:dyDescent="0.25">
       <c r="G50" s="6" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="K50" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="L50" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="M50">
         <v>0.6</v>
       </c>
       <c r="N50" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="P50" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="51" spans="1:16" x14ac:dyDescent="0.25">
       <c r="G51" s="6" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="K51" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="L51" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="M51" s="18">
         <v>56100</v>
       </c>
       <c r="N51" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="O51" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="P51" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="52" spans="1:16" x14ac:dyDescent="0.25">
       <c r="G52" s="6" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="K52" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="L52" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="M52">
         <v>5</v>
       </c>
       <c r="N52" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="P52" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="53" spans="1:16" x14ac:dyDescent="0.25">
       <c r="G53" s="6" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="K53" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="L53" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="M53">
         <v>0.1</v>
       </c>
       <c r="N53" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="P53" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="54" spans="1:16" x14ac:dyDescent="0.25">
       <c r="G54" s="6" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="K54" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="L54" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="M54" s="18">
         <v>0</v>
       </c>
       <c r="N54" t="s">
+        <v>186</v>
+      </c>
+      <c r="O54" t="s">
         <v>187</v>
       </c>
-      <c r="O54" t="s">
-        <v>188</v>
-      </c>
       <c r="P54" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="55" spans="1:16" x14ac:dyDescent="0.25">
       <c r="G55" s="6" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="K55" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="L55" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="M55" s="18">
         <v>300</v>
       </c>
       <c r="N55" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="P55" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="56" spans="1:16" x14ac:dyDescent="0.25">
       <c r="G56" s="6" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="K56" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="L56" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="M56" s="18">
         <v>4</v>
       </c>
       <c r="N56" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="P56" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="57" spans="1:16" x14ac:dyDescent="0.25">
       <c r="G57" s="6" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="L57" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="M57" s="18">
         <v>0</v>
       </c>
       <c r="N57" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="O57" s="15"/>
     </row>
     <row r="58" spans="1:16" x14ac:dyDescent="0.25">
       <c r="G58" s="6" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="L58" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="M58" s="18">
         <v>0</v>
       </c>
       <c r="N58" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="O58" s="15"/>
     </row>
     <row r="59" spans="1:16" x14ac:dyDescent="0.25">
       <c r="G59" s="4" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="L59" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="M59" s="18">
         <v>0</v>
       </c>
       <c r="N59" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="O59" s="15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="60" spans="1:16" x14ac:dyDescent="0.25">
       <c r="G60" s="6" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="L60" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="M60" s="18">
         <v>0</v>
       </c>
       <c r="N60" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="O60" s="15"/>
     </row>
@@ -3807,7 +3810,7 @@
       <c r="E71" s="4"/>
       <c r="F71" s="4"/>
       <c r="G71" s="4" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="H71" s="4"/>
       <c r="I71" s="4"/>
@@ -3830,7 +3833,7 @@
       <c r="E72" s="4"/>
       <c r="F72" s="4"/>
       <c r="G72" s="4" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="H72" s="4"/>
       <c r="I72" s="4"/>
@@ -3853,7 +3856,7 @@
       <c r="E73" s="4"/>
       <c r="F73" s="4"/>
       <c r="G73" s="4" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="H73" s="4"/>
       <c r="I73" s="4"/>
@@ -3876,7 +3879,7 @@
       <c r="E74" s="4"/>
       <c r="F74" s="4"/>
       <c r="G74" s="6" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="H74" s="6"/>
       <c r="I74" s="6"/>
@@ -4161,7 +4164,7 @@
         <v>0</v>
       </c>
       <c r="N96" s="9" t="s">
-        <v>57</v>
+        <v>334</v>
       </c>
       <c r="O96" s="9"/>
     </row>
@@ -4963,6 +4966,9 @@
       <c r="M148" s="13">
         <v>1.6176327916666666</v>
       </c>
+      <c r="N148" t="s">
+        <v>57</v>
+      </c>
       <c r="O148" s="6" t="s">
         <v>135</v>
       </c>
@@ -4978,10 +4984,14 @@
         <v>134</v>
       </c>
       <c r="M149" s="13">
-        <v>3.0774477499999997</v>
+        <f>3.07744775/0.85</f>
+        <v>3.6205267647058825</v>
+      </c>
+      <c r="N149" t="s">
+        <v>334</v>
       </c>
       <c r="O149" s="6" t="s">
-        <v>136</v>
+        <v>335</v>
       </c>
       <c r="P149" s="4" t="s">
         <v>91</v>
@@ -4997,8 +5007,11 @@
       <c r="M150" s="13">
         <v>0.25</v>
       </c>
+      <c r="N150" t="s">
+        <v>59</v>
+      </c>
       <c r="O150" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="P150" s="4" t="s">
         <v>112</v>
@@ -5040,12 +5053,12 @@
         <v>49</v>
       </c>
       <c r="M154" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="156" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A156" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B156" s="1"/>
       <c r="C156" s="1"/>
@@ -5065,13 +5078,13 @@
     </row>
     <row r="157" spans="1:16" x14ac:dyDescent="0.25">
       <c r="L157" s="9" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="M157" s="9">
         <v>0</v>
       </c>
       <c r="N157" s="9" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="O157" s="9" t="s">
         <v>53</v>
@@ -5079,135 +5092,135 @@
     </row>
     <row r="158" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B158" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="L158" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="M158">
         <v>302</v>
       </c>
       <c r="N158" t="s">
+        <v>163</v>
+      </c>
+      <c r="O158" t="s">
         <v>164</v>
       </c>
-      <c r="O158" t="s">
-        <v>165</v>
-      </c>
       <c r="P158" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="159" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B159" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="L159" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="M159">
         <v>197</v>
       </c>
       <c r="N159" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="O159" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="P159" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="160" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B160" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L160" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="M160">
         <v>216</v>
       </c>
       <c r="N160" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="O160" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="P160" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="161" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B161" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="L161" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="M161">
         <v>216</v>
       </c>
       <c r="N161" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="O161" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="162" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B162" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L162" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="M162">
         <v>216</v>
       </c>
       <c r="N162" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="O162" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="163" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B163" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="L163" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="M163">
         <v>216</v>
       </c>
       <c r="N163" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="O163" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="164" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B164" t="s">
+        <v>161</v>
+      </c>
+      <c r="L164" t="s">
         <v>162</v>
-      </c>
-      <c r="L164" t="s">
-        <v>163</v>
       </c>
       <c r="M164">
         <v>216</v>
       </c>
       <c r="N164" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="O164" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="166" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A166" s="1" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B166" s="1"/>
       <c r="C166" s="1"/>
@@ -5227,13 +5240,13 @@
     </row>
     <row r="167" spans="1:16" x14ac:dyDescent="0.25">
       <c r="L167" s="9" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="M167" s="9">
         <v>0</v>
       </c>
       <c r="N167" s="9" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="O167" s="9" t="s">
         <v>53</v>
@@ -5241,13 +5254,13 @@
     </row>
     <row r="168" spans="1:16" x14ac:dyDescent="0.25">
       <c r="L168" s="9" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="M168" s="9">
         <v>0</v>
       </c>
       <c r="N168" s="9" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="O168" s="9" t="s">
         <v>53</v>
@@ -5255,13 +5268,13 @@
     </row>
     <row r="169" spans="1:16" x14ac:dyDescent="0.25">
       <c r="L169" s="9" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="M169" s="9">
         <v>0</v>
       </c>
       <c r="N169" s="9" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="O169" s="9" t="s">
         <v>53</v>
@@ -5269,143 +5282,143 @@
     </row>
     <row r="171" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C171" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D171" t="s">
+        <v>204</v>
+      </c>
+      <c r="E171" t="s">
         <v>205</v>
       </c>
-      <c r="E171" t="s">
-        <v>206</v>
-      </c>
       <c r="F171" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="L171" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="M171" s="25">
         <f>'energy stables'!E24</f>
         <v>3.5302245250431775E-2</v>
       </c>
       <c r="N171" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="O171" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="P171" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="172" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C172" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D172" t="s">
+        <v>204</v>
+      </c>
+      <c r="E172" t="s">
         <v>205</v>
       </c>
-      <c r="E172" t="s">
-        <v>206</v>
-      </c>
       <c r="L172" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="M172" s="24">
         <f>'energy stables'!D26</f>
         <v>308.33833333333342</v>
       </c>
       <c r="N172" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="O172" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="P172" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="173" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C173" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D173" t="s">
+        <v>204</v>
+      </c>
+      <c r="E173" t="s">
         <v>205</v>
       </c>
-      <c r="E173" t="s">
-        <v>206</v>
-      </c>
       <c r="F173" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="L173" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="M173" s="25">
         <f>'energy stables'!E27</f>
         <v>4.1036269430051814E-2</v>
       </c>
       <c r="N173" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="P173" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="175" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C175" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="L175" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="M175" s="24">
         <f>'energy stables'!D29</f>
         <v>170.33333333333331</v>
       </c>
       <c r="N175" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="O175" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="P175" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="176" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C176" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="L176" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="M176" s="24">
         <f>'energy stables'!D31</f>
         <v>332.32333333333338</v>
       </c>
       <c r="N176" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="O176" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="P176" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="177" spans="1:16" x14ac:dyDescent="0.25">
@@ -5413,233 +5426,233 @@
     </row>
     <row r="178" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C178" t="s">
+        <v>235</v>
+      </c>
+      <c r="D178" t="s">
         <v>236</v>
       </c>
-      <c r="D178" t="s">
-        <v>237</v>
-      </c>
       <c r="E178" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="L178" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="M178" s="25">
         <f>(290+1078)/100000</f>
         <v>1.3679999999999999E-2</v>
       </c>
       <c r="N178" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="O178" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="P178" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="179" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C179" t="s">
+        <v>235</v>
+      </c>
+      <c r="D179" t="s">
         <v>236</v>
       </c>
-      <c r="D179" t="s">
-        <v>237</v>
-      </c>
       <c r="E179" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="L179" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="M179" s="25">
         <f>77000/100000</f>
         <v>0.77</v>
       </c>
       <c r="N179" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="P179" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="180" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C180" t="s">
+        <v>235</v>
+      </c>
+      <c r="D180" t="s">
         <v>236</v>
       </c>
-      <c r="D180" t="s">
-        <v>237</v>
-      </c>
       <c r="E180" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="L180" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="M180" s="25">
         <f>(3340+9790)/100000</f>
         <v>0.1313</v>
       </c>
       <c r="N180" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="O180" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="P180" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="182" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C182" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E182" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="L182" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="M182">
         <f>'energy stables'!D49</f>
         <v>3.5</v>
       </c>
       <c r="N182" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="P182" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="183" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C183" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E183" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="L183" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="M183">
         <f>'energy stables'!D50</f>
         <v>12.5</v>
       </c>
       <c r="N183" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="P183" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="184" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C184" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E184" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="L184" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="M184">
         <f>'energy stables'!D51</f>
         <v>34</v>
       </c>
       <c r="N184" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="P184" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="185" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C185" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E185" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="L185" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="M185">
         <f>'energy stables'!D53</f>
         <v>0.04</v>
       </c>
       <c r="N185" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="P185" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="186" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C186" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E186" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="L186" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="M186" s="13">
         <f>'energy stables'!D54</f>
         <v>0.1</v>
       </c>
       <c r="N186" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="P186" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="187" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C187" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E187" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="L187" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="M187" s="13">
         <f>'energy stables'!D55</f>
         <v>0.26</v>
       </c>
       <c r="N187" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="P187" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
   </sheetData>
@@ -5661,7 +5674,7 @@
   <sheetData>
     <row r="3" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B3" s="53" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C3" s="54"/>
       <c r="D3" s="54"/>
@@ -5681,37 +5694,37 @@
     </row>
     <row r="4" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B4" s="51" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="5" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B5" s="27"/>
       <c r="C5" s="30"/>
       <c r="D5" s="46" t="s">
+        <v>207</v>
+      </c>
+      <c r="E5" s="28" t="s">
+        <v>205</v>
+      </c>
+      <c r="F5" s="30" t="s">
+        <v>224</v>
+      </c>
+      <c r="G5" s="29" t="s">
         <v>208</v>
       </c>
-      <c r="E5" s="28" t="s">
-        <v>206</v>
-      </c>
-      <c r="F5" s="30" t="s">
-        <v>225</v>
-      </c>
-      <c r="G5" s="29" t="s">
-        <v>209</v>
-      </c>
       <c r="H5" s="28" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="I5" s="30" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="6" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B6" s="31" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C6" s="44" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D6" s="31">
         <v>150</v>
@@ -5726,10 +5739,10 @@
     </row>
     <row r="7" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B7" s="31" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C7" s="44" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D7" s="31">
         <v>150</v>
@@ -5744,10 +5757,10 @@
     </row>
     <row r="8" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B8" s="31" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C8" s="44" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D8" s="31">
         <v>10500</v>
@@ -5772,10 +5785,10 @@
     </row>
     <row r="10" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B10" s="31" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C10" s="44" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D10" s="31">
         <v>652</v>
@@ -5800,15 +5813,15 @@
         <v>123.33333333333333</v>
       </c>
       <c r="J10" s="26" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="11" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B11" s="31" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C11" s="44" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D11" s="31">
         <v>3</v>
@@ -5836,10 +5849,10 @@
     </row>
     <row r="12" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B12" s="31" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C12" s="44" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D12" s="31">
         <v>40</v>
@@ -5864,15 +5877,15 @@
         <v>10.333333333333332</v>
       </c>
       <c r="J12" s="26" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="13" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B13" s="31" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C13" s="44" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D13" s="31">
         <v>216</v>
@@ -5900,10 +5913,10 @@
     </row>
     <row r="14" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B14" s="31" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C14" s="44" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D14" s="31">
         <v>386</v>
@@ -5926,15 +5939,15 @@
         <v>0</v>
       </c>
       <c r="J14" s="26" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="15" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B15" s="31" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C15" s="44" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D15" s="31">
         <v>216</v>
@@ -5971,10 +5984,10 @@
     </row>
     <row r="17" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B17" s="36" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C17" s="44" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D17" s="36">
         <f>SUM(D10:D15)</f>
@@ -6003,10 +6016,10 @@
     </row>
     <row r="18" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B18" s="31" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C18" s="44" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D18" s="31">
         <v>868</v>
@@ -6061,7 +6074,7 @@
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B20" s="42" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C20" s="45" t="s">
         <v>128</v>
@@ -6079,25 +6092,25 @@
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B22" s="71" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="23" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B23" s="79"/>
       <c r="C23" s="80"/>
       <c r="D23" s="81" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="E23" s="82" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="24" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B24" s="64" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C24" s="65" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D24" s="72">
         <v>0</v>
@@ -6109,10 +6122,10 @@
     </row>
     <row r="25" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B25" s="64" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C25" s="65" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D25" s="72">
         <v>0</v>
@@ -6123,10 +6136,10 @@
     </row>
     <row r="26" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B26" s="64" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C26" s="65" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D26" s="75">
         <f>SUM(E11:E13,E15,H11:H13,H15)/2</f>
@@ -6138,10 +6151,10 @@
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B27" s="64" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C27" s="65" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D27" s="72">
         <v>0</v>
@@ -6159,10 +6172,10 @@
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B29" s="64" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C29" s="65" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D29" s="75">
         <f>SUM(F10,I10)/2</f>
@@ -6174,10 +6187,10 @@
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B30" s="64" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C30" s="65" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D30" s="72">
         <v>0</v>
@@ -6188,10 +6201,10 @@
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B31" s="64" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C31" s="65" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D31" s="75">
         <f>SUM(F11:F13,F15,I11:I13,I15)</f>
@@ -6203,10 +6216,10 @@
     </row>
     <row r="32" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B32" s="66" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C32" s="67" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D32" s="76">
         <v>0</v>
@@ -6217,7 +6230,7 @@
     </row>
     <row r="34" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B34" s="53" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C34" s="54"/>
       <c r="D34" s="54"/>
@@ -6237,69 +6250,69 @@
     </row>
     <row r="35" spans="2:19" x14ac:dyDescent="0.25">
       <c r="J35" s="51" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="36" spans="2:19" x14ac:dyDescent="0.25">
       <c r="J36" s="46" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="K36" s="28"/>
       <c r="L36" s="28"/>
       <c r="M36" s="29" t="s">
+        <v>303</v>
+      </c>
+      <c r="N36" s="29" t="s">
         <v>304</v>
       </c>
-      <c r="N36" s="29" t="s">
+      <c r="O36" s="29" t="s">
         <v>305</v>
       </c>
-      <c r="O36" s="29" t="s">
+      <c r="P36" s="50" t="s">
         <v>306</v>
       </c>
-      <c r="P36" s="50" t="s">
-        <v>307</v>
-      </c>
       <c r="Q36" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="37" spans="2:19" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="51" t="s">
+        <v>253</v>
+      </c>
+      <c r="J37" s="42" t="s">
         <v>254</v>
-      </c>
-      <c r="J37" s="42" t="s">
-        <v>255</v>
       </c>
       <c r="K37" s="14"/>
       <c r="L37" s="14"/>
       <c r="M37" s="59" t="s">
+        <v>299</v>
+      </c>
+      <c r="N37" s="59" t="s">
         <v>300</v>
       </c>
-      <c r="N37" s="59" t="s">
+      <c r="O37" s="59" t="s">
         <v>301</v>
       </c>
-      <c r="O37" s="59" t="s">
+      <c r="P37" s="60" t="s">
         <v>302</v>
       </c>
-      <c r="P37" s="60" t="s">
-        <v>303</v>
-      </c>
       <c r="Q37" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="38" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B38" s="46" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C38" s="29"/>
       <c r="D38" s="29" t="s">
+        <v>247</v>
+      </c>
+      <c r="E38" s="50" t="s">
         <v>248</v>
       </c>
-      <c r="E38" s="50" t="s">
-        <v>249</v>
-      </c>
       <c r="J38" s="31" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="K38" s="4"/>
       <c r="L38" s="4"/>
@@ -6316,14 +6329,14 @@
         <v>242</v>
       </c>
       <c r="Q38" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="R38" s="58"/>
       <c r="S38" s="58"/>
     </row>
     <row r="39" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B39" s="31" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C39" s="4"/>
       <c r="D39" s="4">
@@ -6333,7 +6346,7 @@
         <v>0.4</v>
       </c>
       <c r="J39" s="31" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="K39" s="4"/>
       <c r="L39" s="4"/>
@@ -6347,17 +6360,17 @@
         <v>9.6</v>
       </c>
       <c r="P39" s="32" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="Q39" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="R39" s="58"/>
       <c r="S39" s="58"/>
     </row>
     <row r="40" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B40" s="31" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C40" s="4"/>
       <c r="D40" s="4">
@@ -6367,7 +6380,7 @@
         <v>0.28000000000000003</v>
       </c>
       <c r="J40" s="31" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="K40" s="4"/>
       <c r="L40" s="4"/>
@@ -6384,14 +6397,14 @@
         <v>43.2</v>
       </c>
       <c r="Q40" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="R40" s="58"/>
       <c r="S40" s="58"/>
     </row>
     <row r="41" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B41" s="31" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C41" s="4"/>
       <c r="D41" s="4">
@@ -6401,7 +6414,7 @@
         <v>0.06</v>
       </c>
       <c r="J41" s="31" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="K41" s="4"/>
       <c r="L41" s="4"/>
@@ -6418,14 +6431,14 @@
         <v>340</v>
       </c>
       <c r="Q41" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="R41" s="58"/>
       <c r="S41" s="58"/>
     </row>
     <row r="42" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B42" s="31" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="C42" s="4"/>
       <c r="D42" s="4">
@@ -6435,7 +6448,7 @@
         <v>0.04</v>
       </c>
       <c r="J42" s="31" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="K42" s="4"/>
       <c r="L42" s="4"/>
@@ -6449,17 +6462,17 @@
         <v>4.2</v>
       </c>
       <c r="P42" s="32" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="Q42" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="R42" s="58"/>
       <c r="S42" s="58"/>
     </row>
     <row r="43" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B43" s="42" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C43" s="14"/>
       <c r="D43" s="14">
@@ -6491,41 +6504,41 @@
     </row>
     <row r="44" spans="2:19" x14ac:dyDescent="0.25">
       <c r="C44" s="68" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="D44" s="69">
         <f>D39*33+E39*26</f>
         <v>1660.4</v>
       </c>
       <c r="E44" s="70" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="J44" s="31" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="K44" s="4"/>
       <c r="L44" s="4"/>
       <c r="M44" s="4" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="N44" s="4">
         <v>4</v>
       </c>
       <c r="O44" s="4" t="s">
+        <v>270</v>
+      </c>
+      <c r="P44" s="32" t="s">
         <v>271</v>
       </c>
-      <c r="P44" s="32" t="s">
-        <v>272</v>
-      </c>
       <c r="Q44" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="R44" s="58"/>
       <c r="S44" s="58"/>
     </row>
     <row r="45" spans="2:19" x14ac:dyDescent="0.25">
       <c r="J45" s="31" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="K45" s="4"/>
       <c r="L45" s="4"/>
@@ -6539,20 +6552,20 @@
         <v>0.7</v>
       </c>
       <c r="P45" s="32" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="Q45" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="R45" s="58"/>
       <c r="S45" s="58"/>
     </row>
     <row r="46" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B46" s="71" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="J46" s="31" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="K46" s="4"/>
       <c r="L46" s="4"/>
@@ -6566,10 +6579,10 @@
         <v>87</v>
       </c>
       <c r="P46" s="32" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="Q46" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="R46" s="58"/>
       <c r="S46" s="58"/>
@@ -6578,16 +6591,16 @@
       <c r="B47" s="27"/>
       <c r="C47" s="28"/>
       <c r="D47" s="86" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="E47" s="28" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="F47" s="28"/>
       <c r="G47" s="28"/>
       <c r="H47" s="30"/>
       <c r="J47" s="31" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="K47" s="4"/>
       <c r="L47" s="4"/>
@@ -6598,13 +6611,13 @@
         <v>15</v>
       </c>
       <c r="O47" s="4" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="P47" s="32" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="Q47" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="R47" s="58"/>
       <c r="S47" s="58"/>
@@ -6613,22 +6626,22 @@
       <c r="B48" s="42"/>
       <c r="C48" s="14"/>
       <c r="D48" s="87" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="E48" s="14" t="s">
         <v>26</v>
       </c>
       <c r="F48" s="83" t="s">
+        <v>151</v>
+      </c>
+      <c r="G48" s="83" t="s">
         <v>152</v>
       </c>
-      <c r="G48" s="83" t="s">
-        <v>153</v>
-      </c>
       <c r="H48" s="84" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="J48" s="31" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="K48" s="4"/>
       <c r="L48" s="4"/>
@@ -6642,20 +6655,20 @@
         <v>1</v>
       </c>
       <c r="P48" s="32" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="Q48" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="R48" s="58"/>
       <c r="S48" s="58"/>
     </row>
     <row r="49" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B49" s="85" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C49" s="28" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="D49" s="88">
         <f>D42</f>
@@ -6674,7 +6687,7 @@
         <v>0</v>
       </c>
       <c r="J49" s="46" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="K49" s="29"/>
       <c r="L49" s="29"/>
@@ -6691,17 +6704,17 @@
         <v>1252</v>
       </c>
       <c r="Q49" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="R49" s="58"/>
       <c r="S49" s="58"/>
     </row>
     <row r="50" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B50" s="31" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="D50" s="88">
         <f>D39*0.25</f>
@@ -6723,7 +6736,7 @@
         <v>20</v>
       </c>
       <c r="J50" s="31" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="K50" s="4"/>
       <c r="L50" s="4"/>
@@ -6744,10 +6757,10 @@
     </row>
     <row r="51" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B51" s="31" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="D51" s="89">
         <f>D39-D49-D50</f>
@@ -6766,7 +6779,7 @@
         <v>100</v>
       </c>
       <c r="J51" s="61" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="K51" s="63"/>
       <c r="L51" s="63"/>
@@ -6787,7 +6800,7 @@
         <v>34</v>
       </c>
       <c r="Q51" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="R51" s="58"/>
       <c r="S51" s="58"/>
@@ -6801,7 +6814,7 @@
       <c r="G52" s="72"/>
       <c r="H52" s="74"/>
       <c r="J52" s="55" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K52" s="56"/>
       <c r="L52" s="56"/>
@@ -6815,18 +6828,18 @@
         <v>87</v>
       </c>
       <c r="P52" s="57" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="Q52" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="53" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B53" s="64" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="D53" s="88">
         <f>E42</f>
@@ -6845,32 +6858,32 @@
         <v>0</v>
       </c>
       <c r="J53" s="31" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="K53" s="4"/>
       <c r="L53" s="4"/>
       <c r="M53" s="4" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="N53" s="4" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="O53" s="4" t="s">
         <v>87</v>
       </c>
       <c r="P53" s="32" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="Q53" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="54" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B54" s="31" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="D54" s="90">
         <f>E39*0.25</f>
@@ -6892,32 +6905,32 @@
         <v>20.000000000000018</v>
       </c>
       <c r="J54" s="31" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="K54" s="4"/>
       <c r="L54" s="4"/>
       <c r="M54" s="4" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="N54" s="4" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="O54" s="4" t="s">
         <v>87</v>
       </c>
       <c r="P54" s="32" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="Q54" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="55" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B55" s="42" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C55" s="14" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="D55" s="91">
         <f>E39-D53-D54</f>
@@ -6936,27 +6949,27 @@
         <v>100</v>
       </c>
       <c r="J55" s="31" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="K55" s="4"/>
       <c r="L55" s="4"/>
       <c r="M55" s="4" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="N55" s="4"/>
       <c r="O55" s="4" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="P55" s="32" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="Q55" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="56" spans="2:19" x14ac:dyDescent="0.25">
       <c r="J56" s="42" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="K56" s="14"/>
       <c r="L56" s="14"/>
@@ -7008,7 +7021,7 @@
   <sheetData>
     <row r="3" spans="5:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="F3">
         <v>90</v>
@@ -7025,7 +7038,7 @@
     </row>
     <row r="4" spans="5:20" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E4" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="F4">
         <v>654</v>
@@ -7034,15 +7047,15 @@
         <v>80</v>
       </c>
       <c r="H4" t="s">
+        <v>260</v>
+      </c>
+      <c r="I4" t="s">
         <v>261</v>
-      </c>
-      <c r="I4" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="5" spans="5:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E5" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="F5">
         <v>11</v>
@@ -7051,66 +7064,66 @@
         <v>12</v>
       </c>
       <c r="H5" t="s">
+        <v>263</v>
+      </c>
+      <c r="I5" t="s">
         <v>264</v>
-      </c>
-      <c r="I5" t="s">
-        <v>265</v>
       </c>
     </row>
     <row r="6" spans="5:20" x14ac:dyDescent="0.25">
       <c r="E6" t="s">
+        <v>292</v>
+      </c>
+      <c r="F6" t="s">
         <v>293</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>294</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>295</v>
       </c>
-      <c r="H6" t="s">
+      <c r="I6" t="s">
         <v>296</v>
-      </c>
-      <c r="I6" t="s">
-        <v>297</v>
       </c>
     </row>
     <row r="7" spans="5:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E7" t="s">
+        <v>255</v>
+      </c>
+      <c r="G7" t="s">
+        <v>265</v>
+      </c>
+      <c r="I7" t="s">
+        <v>266</v>
+      </c>
+      <c r="O7" t="s">
+        <v>267</v>
+      </c>
+      <c r="S7" t="s">
         <v>256</v>
-      </c>
-      <c r="G7" t="s">
-        <v>266</v>
-      </c>
-      <c r="I7" t="s">
-        <v>267</v>
-      </c>
-      <c r="O7" t="s">
-        <v>268</v>
-      </c>
-      <c r="S7" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="8" spans="5:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E8" t="s">
+        <v>268</v>
+      </c>
+      <c r="H8" t="s">
         <v>269</v>
-      </c>
-      <c r="H8" t="s">
-        <v>270</v>
       </c>
       <c r="K8">
         <v>4</v>
       </c>
       <c r="P8" t="s">
+        <v>270</v>
+      </c>
+      <c r="T8" t="s">
         <v>271</v>
-      </c>
-      <c r="T8" t="s">
-        <v>272</v>
       </c>
     </row>
     <row r="9" spans="5:20" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E9" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="H9">
         <v>79</v>
@@ -7119,15 +7132,15 @@
         <v>7</v>
       </c>
       <c r="P9" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="T9" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="10" spans="5:20" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E10" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="H10" t="s">
         <v>87</v>
@@ -7139,12 +7152,12 @@
         <v>87</v>
       </c>
       <c r="T10" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="11" spans="5:20" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E11" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="H11">
         <v>38</v>
@@ -7153,15 +7166,15 @@
         <v>15</v>
       </c>
       <c r="P11" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="T11" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="12" spans="5:20" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E12" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="H12">
         <v>164</v>
@@ -7170,15 +7183,15 @@
         <v>66</v>
       </c>
       <c r="P12" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="T12" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="13" spans="5:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E13" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="H13">
         <v>2433</v>
@@ -7187,7 +7200,7 @@
         <v>689</v>
       </c>
       <c r="P13" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="T13">
         <v>1252</v>
@@ -7195,7 +7208,7 @@
     </row>
     <row r="14" spans="5:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E14" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="H14">
         <v>1441</v>
@@ -7204,7 +7217,7 @@
         <v>689</v>
       </c>
       <c r="P14" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="T14">
         <v>1218</v>
@@ -7212,47 +7225,47 @@
     </row>
     <row r="15" spans="5:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E15" t="s">
+        <v>282</v>
+      </c>
+      <c r="L15" t="s">
         <v>283</v>
       </c>
-      <c r="L15" t="s">
+      <c r="Q15" t="s">
         <v>284</v>
-      </c>
-      <c r="Q15" t="s">
-        <v>285</v>
       </c>
     </row>
     <row r="16" spans="5:20" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E16" t="s">
+        <v>285</v>
+      </c>
+      <c r="H16" t="s">
         <v>286</v>
       </c>
-      <c r="H16" t="s">
-        <v>287</v>
-      </c>
       <c r="K16" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="P16" t="s">
         <v>87</v>
       </c>
       <c r="T16" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="17" spans="5:20" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E17" t="s">
+        <v>287</v>
+      </c>
+      <c r="H17" t="s">
         <v>288</v>
       </c>
-      <c r="H17" t="s">
+      <c r="K17" t="s">
         <v>289</v>
       </c>
-      <c r="K17" t="s">
+      <c r="P17" t="s">
         <v>290</v>
       </c>
-      <c r="P17" t="s">
+      <c r="T17" t="s">
         <v>291</v>
-      </c>
-      <c r="T17" t="s">
-        <v>292</v>
       </c>
     </row>
   </sheetData>
@@ -7271,47 +7284,47 @@
   <sheetData>
     <row r="3" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C3" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="F3" s="49" t="s">
+        <v>303</v>
+      </c>
+      <c r="G3" s="49" t="s">
         <v>304</v>
       </c>
-      <c r="G3" s="49" t="s">
+      <c r="H3" s="49" t="s">
         <v>305</v>
       </c>
-      <c r="H3" s="49" t="s">
+      <c r="I3" s="49" t="s">
         <v>306</v>
       </c>
-      <c r="I3" s="49" t="s">
-        <v>307</v>
-      </c>
       <c r="J3" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="4" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="F4" t="s">
+        <v>299</v>
+      </c>
+      <c r="G4" t="s">
         <v>300</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>301</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>302</v>
       </c>
-      <c r="I4" t="s">
-        <v>303</v>
-      </c>
       <c r="J4" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="5" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="F5">
         <v>90</v>
@@ -7326,12 +7339,12 @@
         <v>242</v>
       </c>
       <c r="J5" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="6" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="F6">
         <v>654</v>
@@ -7343,15 +7356,15 @@
         <v>9.6</v>
       </c>
       <c r="I6" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="J6" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="7" spans="3:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="F7">
         <v>11</v>
@@ -7366,12 +7379,12 @@
         <v>43.2</v>
       </c>
       <c r="J7" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="8" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="F8">
         <v>244</v>
@@ -7386,12 +7399,12 @@
         <v>340</v>
       </c>
       <c r="J8" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="9" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="F9">
         <v>992</v>
@@ -7403,35 +7416,35 @@
         <v>4.2</v>
       </c>
       <c r="I9" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="J9" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="10" spans="3:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
+        <v>268</v>
+      </c>
+      <c r="F10" t="s">
         <v>269</v>
-      </c>
-      <c r="F10" t="s">
-        <v>270</v>
       </c>
       <c r="G10">
         <v>4</v>
       </c>
       <c r="H10" t="s">
+        <v>270</v>
+      </c>
+      <c r="I10" t="s">
         <v>271</v>
       </c>
-      <c r="I10" t="s">
-        <v>272</v>
-      </c>
       <c r="J10" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="11" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F11">
         <v>79</v>
@@ -7443,15 +7456,15 @@
         <v>0.7</v>
       </c>
       <c r="I11" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="J11" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="12" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C12" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F12" t="s">
         <v>87</v>
@@ -7463,15 +7476,15 @@
         <v>87</v>
       </c>
       <c r="I12" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="J12" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="13" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C13" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F13">
         <v>38</v>
@@ -7480,18 +7493,18 @@
         <v>15</v>
       </c>
       <c r="H13" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="I13" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="J13" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="14" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C14" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="F14">
         <v>164</v>
@@ -7503,15 +7516,15 @@
         <v>1</v>
       </c>
       <c r="I14" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="J14" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="15" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C15" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F15">
         <v>2433</v>
@@ -7526,12 +7539,12 @@
         <v>1252</v>
       </c>
       <c r="J15" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="16" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C16" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="F16">
         <v>1441</v>
@@ -7546,12 +7559,12 @@
         <v>1218</v>
       </c>
       <c r="J16" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="17" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C17" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="F17">
         <v>23</v>
@@ -7563,72 +7576,72 @@
         <v>87</v>
       </c>
       <c r="I17" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="J17" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="18" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C18" t="s">
+        <v>285</v>
+      </c>
+      <c r="F18" t="s">
         <v>286</v>
       </c>
-      <c r="F18" t="s">
-        <v>287</v>
-      </c>
       <c r="G18" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="H18" t="s">
         <v>87</v>
       </c>
       <c r="I18" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="J18" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="19" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C19" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="F19" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="G19" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="H19" t="s">
         <v>87</v>
       </c>
       <c r="I19" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="J19" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="20" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C20" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="F20" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="H20" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="I20" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="J20" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="21" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C21" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="F21">
         <v>1998</v>
@@ -7643,7 +7656,7 @@
         <v>2008</v>
       </c>
       <c r="J21" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
   </sheetData>
@@ -7659,62 +7672,62 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="17" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="17" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="48" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="48" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated share oil for grain dryers
</commit_message>
<xml_diff>
--- a/data/default/MachineryAndEnergyMgmt.xlsx
+++ b/data/default/MachineryAndEnergyMgmt.xlsx
@@ -477,7 +477,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1017" uniqueCount="359">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1020" uniqueCount="361">
   <si>
     <t>f_crop</t>
   </si>
@@ -1732,6 +1732,12 @@
   </si>
   <si>
     <t>Törner &amp; Norup 2009, p.11</t>
+  </si>
+  <si>
+    <t>Energimyndigheten. Statistikdatabas. Jordbrukets energianvändning</t>
+  </si>
+  <si>
+    <t>70% of dryers used oil as fuel and consumed 165 GWh oil year 2021</t>
   </si>
 </sst>
 </file>
@@ -2141,7 +2147,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="95">
+  <cellXfs count="94">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -2240,7 +2246,6 @@
     <xf numFmtId="2" fontId="23" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3223,16 +3228,22 @@
         <v>348</v>
       </c>
       <c r="H36" s="6" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="M36" s="6" t="s">
         <v>154</v>
       </c>
-      <c r="N36" s="94">
-        <v>10</v>
+      <c r="N36" s="18">
+        <v>70</v>
       </c>
       <c r="O36" t="s">
         <v>128</v>
+      </c>
+      <c r="P36" t="s">
+        <v>360</v>
+      </c>
+      <c r="Q36" t="s">
+        <v>359</v>
       </c>
     </row>
     <row r="37" spans="1:17" x14ac:dyDescent="0.25">
@@ -3240,16 +3251,19 @@
         <v>348</v>
       </c>
       <c r="H37" s="6" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="M37" s="6" t="s">
         <v>154</v>
       </c>
-      <c r="N37" s="94">
-        <v>90</v>
+      <c r="N37" s="18">
+        <v>30</v>
       </c>
       <c r="O37" t="s">
         <v>128</v>
+      </c>
+      <c r="Q37" t="s">
+        <v>359</v>
       </c>
     </row>
     <row r="38" spans="1:17" x14ac:dyDescent="0.25">

</xml_diff>